<commit_message>
doc(Architecture):Simplification du chemin des fichiers epub et mise à jour du journal de travail
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_MatiasDenis.xlsx
+++ b/Journal-de-Travail_MatiasDenis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\05-repertoires-ict-ssd (2022)\Deuxième année\P_AppMobile\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projet_README\P_AppMobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F20068F-0D8A-4074-81DA-D972774F8FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9DA9768-39E5-4E43-AB51-71216A74308F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="33705" yWindow="1620" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>Création de la maquette high-fidelity sur Figma, regroupant les fonctionnalités demandées dans le cahier des charges.</t>
+  </si>
+  <si>
+    <t>Absence - Maladie.</t>
   </si>
 </sst>
 </file>
@@ -1048,7 +1051,7 @@
                   <c:v>1.0416666666666666E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>1.7361111111111112E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2008,7 +2011,7 @@
       </c>
       <c r="C3" s="25" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 3 heurs 15 minutes</v>
+        <v>0 jours 6 heurs 40 minutes</v>
       </c>
       <c r="D3" s="25"/>
       <c r="E3" s="3"/>
@@ -2023,15 +2026,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="25">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>180</v>
+        <v>360</v>
       </c>
       <c r="D4" s="25">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="E4" s="52">
         <f>SUM(C4:D4)</f>
-        <v>195</v>
+        <v>400</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2116,11 +2119,21 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="18"/>
-      <c r="B9" s="40"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="48"/>
+      <c r="B9" s="40">
+        <v>46055</v>
+      </c>
+      <c r="C9" s="36">
+        <v>3</v>
+      </c>
+      <c r="D9" s="44">
+        <v>25</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="48" t="s">
+        <v>32</v>
+      </c>
       <c r="G9" s="20"/>
       <c r="M9" t="s">
         <v>4</v>
@@ -8253,7 +8266,7 @@
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B11">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C11,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C11" s="51" t="str">
         <f>'Journal de travail'!M15</f>
@@ -8261,7 +8274,7 @@
       </c>
       <c r="D11" s="45">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.7361111111111112E-2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -8270,7 +8283,7 @@
       </c>
       <c r="D12" s="46">
         <f>SUM(D4:D11)</f>
-        <v>5.2083333333333329E-2</v>
+        <v>6.9444444444444448E-2</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -8283,14 +8296,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8501,23 +8512,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="26488081-7094-48e3-a435-bbb366c5709a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="eb2b4dc0-5538-4988-a426-1e3bf3687743">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
-    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
-    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
-    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8542,9 +8550,14 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be0d3259-a7ce-4623-88ec-81594dfcbc1c"/>
+    <ds:schemaRef ds:uri="99ffe1f3-7857-457f-add0-5bdef636f38d"/>
+    <ds:schemaRef ds:uri="26488081-7094-48e3-a435-bbb366c5709a"/>
+    <ds:schemaRef ds:uri="eb2b4dc0-5538-4988-a426-1e3bf3687743"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
doc(JdT): mise à jour du journal de travail
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_MatiasDenis.xlsx
+++ b/Journal-de-Travail_MatiasDenis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projet_README\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C32DFDC-36AC-49CA-9C46-E8AB8E886B26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4DB2D6-7938-485D-8819-35B3772D5A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32040" yWindow="1020" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -186,6 +186,29 @@
   </si>
   <si>
     <t>Correction de l'arborescence des fichiers et importation réussie de la bibliothèque complète (6 livres) en format binaire (MEDIUMBLOB) dans MySQL via le BookSeeder.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Refactorisation complète du </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>BooksController</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pour répondre aux exigences du projet ReadME : implémentation du tri par date d'ajout pour la liste des livres , intégration du support pour le contenu binaire (BLOB) dans la méthode d'affichage et nettoyage des champs obsolètes (pdf_link, image_path).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1085,7 +1108,7 @@
                   <c:v>0.10416666666666667</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.1666666666666664E-2</c:v>
+                  <c:v>6.25E-2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2063,7 +2086,7 @@
       </c>
       <c r="C3" s="25" t="str">
         <f>INT(E4/1440)&amp;" jours "&amp;INT(MOD(E4/1440,1)*24)&amp;" heurs "&amp;INT(MOD(MOD(E4/1440,1)*24,1)*60)&amp;" minutes"</f>
-        <v>0 jours 9 heurs 9 minutes</v>
+        <v>0 jours 9 heurs 40 minutes</v>
       </c>
       <c r="D3" s="25"/>
       <c r="E3" s="3"/>
@@ -2082,11 +2105,11 @@
       </c>
       <c r="D4" s="25">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>130</v>
+        <v>160</v>
       </c>
       <c r="E4" s="52">
         <f>SUM(C4:D4)</f>
-        <v>550</v>
+        <v>580</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="7"/>
@@ -2275,13 +2298,21 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" ht="63">
       <c r="A13" s="18"/>
-      <c r="B13" s="40"/>
+      <c r="B13" s="40">
+        <v>46062</v>
+      </c>
       <c r="C13" s="36"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="48"/>
+      <c r="D13" s="44">
+        <v>30</v>
+      </c>
+      <c r="E13" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>36</v>
+      </c>
       <c r="G13" s="20"/>
       <c r="M13" t="s">
         <v>8</v>
@@ -8246,7 +8277,7 @@
       </c>
       <c r="B5">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Analyse!C5,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C5" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -8254,7 +8285,7 @@
       </c>
       <c r="D5" s="45">
         <f t="shared" ref="D5:D11" si="0">(A5+B5)/1440</f>
-        <v>4.1666666666666664E-2</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -8363,7 +8394,7 @@
       </c>
       <c r="D12" s="46">
         <f>SUM(D4:D11)</f>
-        <v>0.1736111111111111</v>
+        <v>0.19444444444444445</v>
       </c>
     </row>
     <row r="14" spans="1:4">

</xml_diff>